<commit_message>
Laying groundwork for incorporating new moodys data
Archived previous data outputs folder and imported new moodys data.  Require modifying the naics-based-industry-projection file in data/raw to see new data in re-run
</commit_message>
<xml_diff>
--- a/data/processed/sam_auto_dashboard_2025_Q1/custom_table_output/segment_stage_projection_change.xlsx
+++ b/data/processed/sam_auto_dashboard_2025_Q1/custom_table_output/segment_stage_projection_change.xlsx
@@ -603,7 +603,7 @@
         <v>20928.03175770727</v>
       </c>
       <c r="C2" s="5">
-        <v>-1081.333042735339</v>
+        <v>-878.5084842286997</v>
       </c>
       <c r="D2" s="5">
         <v>-1318.236612005687</v>
@@ -623,7 +623,7 @@
         <v>45205</v>
       </c>
       <c r="C3" s="5">
-        <v>-5077.79540316463</v>
+        <v>-4858.133914923368</v>
       </c>
       <c r="D3" s="5">
         <v>-4163.500132041547</v>
@@ -643,7 +643,7 @@
         <v>6089.070013066867</v>
       </c>
       <c r="C4" s="5">
-        <v>17.23242967966507</v>
+        <v>33.4350168593819</v>
       </c>
       <c r="D4" s="5">
         <v>-108.7435517749173</v>
@@ -663,7 +663,7 @@
         <v>8874.553681709274</v>
       </c>
       <c r="C5" s="5">
-        <v>-1246.759581817736</v>
+        <v>-1181.762009322606</v>
       </c>
       <c r="D5" s="5">
         <v>-1316.59722711072</v>
@@ -683,7 +683,7 @@
         <v>14602.46596485234</v>
       </c>
       <c r="C6" s="5">
-        <v>-461.0157953786966</v>
+        <v>-402.1281516805338</v>
       </c>
       <c r="D6" s="5">
         <v>-597.8913766742917</v>
@@ -703,7 +703,7 @@
         <v>5948.051175681669</v>
       </c>
       <c r="C7" s="5">
-        <v>-85.59174075886585</v>
+        <v>-74.07271016237701</v>
       </c>
       <c r="D7" s="5">
         <v>-93.13266577734885</v>
@@ -723,7 +723,7 @@
         <v>1012.884668579939</v>
       </c>
       <c r="C8" s="5">
-        <v>27.76964104335434</v>
+        <v>16.18738774641247</v>
       </c>
       <c r="D8" s="5">
         <v>12.49068975850969</v>
@@ -743,7 +743,7 @@
         <v>166447</v>
       </c>
       <c r="C9" s="5">
-        <v>6714.887480545469</v>
+        <v>7041.251589417894</v>
       </c>
       <c r="D9" s="5">
         <v>1171.666182779969</v>
@@ -763,7 +763,7 @@
         <v>116571</v>
       </c>
       <c r="C10" s="5">
-        <v>631.5096448161639</v>
+        <v>1277.071798159406</v>
       </c>
       <c r="D10" s="5">
         <v>1378.862947420042</v>
@@ -783,7 +783,7 @@
         <v>72444</v>
       </c>
       <c r="C11" s="5">
-        <v>1073.834184328065</v>
+        <v>934.9594199421263</v>
       </c>
       <c r="D11" s="5">
         <v>1782.835600903825</v>
@@ -803,7 +803,7 @@
         <v>223902.0572615974</v>
       </c>
       <c r="C12" s="8">
-        <v>3885.189390577842</v>
+        <v>4554.402638629428</v>
       </c>
       <c r="D12" s="8">
         <v>-2250.444560804521</v>
@@ -858,7 +858,7 @@
         <v>234220</v>
       </c>
       <c r="C2" s="5">
-        <v>-3372.451574020408</v>
+        <v>-2646.10269682185</v>
       </c>
       <c r="D2" s="5">
         <v>-1001.801583717694</v>
@@ -878,7 +878,7 @@
         <v>167459.8846685799</v>
       </c>
       <c r="C3" s="5">
-        <v>6742.657121588825</v>
+        <v>7057.438977164304</v>
       </c>
       <c r="D3" s="5">
         <v>1184.156872538471</v>
@@ -898,7 +898,7 @@
         <v>56442.17259301741</v>
       </c>
       <c r="C4" s="5">
-        <v>-2857.467731010969</v>
+        <v>-2503.036338534832</v>
       </c>
       <c r="D4" s="5">
         <v>-3434.601433342956</v>
@@ -918,7 +918,7 @@
         <v>223902.0572615974</v>
       </c>
       <c r="C5" s="8">
-        <v>3885.189390577842</v>
+        <v>4554.402638629428</v>
       </c>
       <c r="D5" s="8">
         <v>-2250.444560804521</v>

</xml_diff>